<commit_message>
Correct device names: iPhone Air, Galaxy Z Fold 8 / Z Flip 8
</commit_message>
<xml_diff>
--- a/Store_Performance_Tracker.xlsx
+++ b/Store_Performance_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jer_2\store-tracker-v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843EFF93-5950-4976-95F6-4AA9BBC88111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BCEF57E-6A81-4BA0-9D3A-75ED56BA94D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="30765" yWindow="855" windowWidth="21600" windowHeight="14835" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -202,7 +202,7 @@
     <t>Expert 03</t>
   </si>
   <si>
-    <t>iPhone 17 Air</t>
+    <t>iPhone Air</t>
   </si>
   <si>
     <t>Expert 04</t>
@@ -256,10 +256,10 @@
     <t>Expert 12</t>
   </si>
   <si>
-    <t>Galaxy Z Fold 7</t>
-  </si>
-  <si>
-    <t>Galaxy Z Flip 7</t>
+    <t>Galaxy Z Fold 8</t>
+  </si>
+  <si>
+    <t>Galaxy Z Flip 8</t>
   </si>
   <si>
     <t>Galaxy A37</t>
@@ -5674,7 +5674,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-3BBE-4C02-B092-F8866CA66B1D}"/>
+              <c16:uniqueId val="{00000000-486B-4095-A6BF-046366D790EA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -5910,7 +5910,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-3BBE-4C02-B092-F8866CA66B1D}"/>
+              <c16:uniqueId val="{00000001-486B-4095-A6BF-046366D790EA}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
Remove frozen panes (iOS duplicate-header rendering) and reset workbook open state to Dashboard
</commit_message>
<xml_diff>
--- a/Store_Performance_Tracker.xlsx
+++ b/Store_Performance_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jer_2\store-tracker-v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E96C756D-3675-49AD-97D8-36538EAA34BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED4CEEFB-E190-4A7C-B99E-094991878FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="30765" yWindow="855" windowWidth="21600" windowHeight="14835" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30765" yWindow="855" windowWidth="21600" windowHeight="14835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -5931,7 +5931,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-506E-49B4-9C7C-D27311C961B1}"/>
+              <c16:uniqueId val="{00000000-DC8E-4472-818E-720CE2F4BADD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6167,7 +6167,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-506E-49B4-9C7C-D27311C961B1}"/>
+              <c16:uniqueId val="{00000001-DC8E-4472-818E-720CE2F4BADD}"/>
             </c:ext>
           </c:extLst>
         </c:ser>

</xml_diff>

<commit_message>
Add standalone web dashboard; revert row/column hiding in Excel
The Excel dashboard's layout is unchanged on desktop, but hiding the rows and
columns outside the design area backfired: hidden rows do not disappear, they
collapse into a visible discontinuity (row headers jumping 46 -> 121, columns
A..Q then DA) that reads as a broken sheet on mobile. Only the three chart
helper columns stay hidden now, which plotVisOnly=0 already accounts for.

A spreadsheet is the wrong surface for reading a dashboard on a phone, so the
reporting layer moves to a self-contained HTML page: same numbers, tooltips on
every mark, pace vs required pace, per-metric heatmap, light/dark themes and a
table view so nothing is encoded in colour alone.

Also renames the leaderboard screenshot to the name the README already
referenced, so the two stop drifting apart.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LEDjB4CVqBST3MAsGzHH1f
</commit_message>
<xml_diff>
--- a/Store_Performance_Tracker.xlsx
+++ b/Store_Performance_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jer_2\store-tracker-v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3B96FC9-D844-465F-922E-9ED9249CD547}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACBDC7F-0C7F-4856-8BFF-2131C21B4CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30765" yWindow="855" windowWidth="21600" windowHeight="14835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5990,7 +5990,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C504-4BC9-94DF-A8DBD5484080}"/>
+              <c16:uniqueId val="{00000000-CBA7-4B7B-865B-8D0FE2C2A621}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6226,7 +6226,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-C504-4BC9-94DF-A8DBD5484080}"/>
+              <c16:uniqueId val="{00000001-CBA7-4B7B-865B-8D0FE2C2A621}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6689,8 +6689,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DA120"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:V46"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.140625" customWidth="1"/>
     <col min="2" max="4" width="11" customWidth="1"/>
@@ -6701,9 +6701,7 @@
     <col min="13" max="13" width="1.5703125" customWidth="1"/>
     <col min="14" max="16" width="11" customWidth="1"/>
     <col min="17" max="17" width="2.140625" customWidth="1"/>
-    <col min="18" max="22" width="13" hidden="1" customWidth="1"/>
-    <col min="23" max="104" width="13" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="105" max="105" width="9.140625" collapsed="1"/>
+    <col min="20" max="22" width="13" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -8074,80 +8072,6 @@
       <c r="P46" s="1"/>
       <c r="Q46" s="1"/>
     </row>
-    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="49" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="50" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="51" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="52" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="53" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="54" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="55" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="56" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="57" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="58" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="59" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="60" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="61" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="62" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="63" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="64" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="65" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="66" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="67" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="68" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="69" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="70" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="71" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="72" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="73" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="74" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="75" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="76" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="77" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="78" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="79" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="80" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="81" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="82" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="83" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="84" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="85" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="86" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="87" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="88" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="89" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="90" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="91" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="92" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="93" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="94" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="95" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="96" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="97" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="98" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="99" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="100" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="101" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="102" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="103" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="104" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="105" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="106" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="107" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="108" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="109" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="110" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="111" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="112" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="113" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="114" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="115" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="116" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="117" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="118" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="119" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="120" hidden="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="44">
     <mergeCell ref="B29:L29"/>

</xml_diff>

<commit_message>
Show the web dashboard in the README; un-clip the leaderboard screenshot
The README described the standalone web page but never showed it, so the one
part of the project that is actually pleasant to look at on a phone was
invisible to anyone browsing the repo. Adds a desktop capture of it.

The leaderboard screenshot was cropped at column F, which cut the row-2
mock-data notice mid-word, ending at 'store numbers appear in t'. That notice
is the privacy disclosure, and a truncated one in a README image is worse than
none. The text overflows to roughly column G, so the capture range now runs
A1:G16.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LEDjB4CVqBST3MAsGzHH1f
</commit_message>
<xml_diff>
--- a/Store_Performance_Tracker.xlsx
+++ b/Store_Performance_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jer_2\store-tracker-v2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACBDC7F-0C7F-4856-8BFF-2131C21B4CF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB26559-1047-415F-BC30-619A28652D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="30765" yWindow="855" windowWidth="21600" windowHeight="14835" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5661,30 +5661,35 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="166" fontId="0" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="20" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="16" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="25" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="25" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
+    <xf numFmtId="3" fontId="22" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -5698,28 +5703,23 @@
     <xf numFmtId="0" fontId="21" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="22" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="25" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="8" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -6734,25 +6734,25 @@
     </row>
     <row r="2" spans="1:22" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
-      <c r="B2" s="42" t="s">
+      <c r="B2" s="45" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="34"/>
-      <c r="D2" s="34"/>
-      <c r="E2" s="34"/>
-      <c r="F2" s="34"/>
-      <c r="G2" s="34"/>
-      <c r="H2" s="34"/>
-      <c r="I2" s="34"/>
+      <c r="C2" s="32"/>
+      <c r="D2" s="32"/>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
       <c r="L2" s="1"/>
-      <c r="M2" s="47" t="s">
+      <c r="M2" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="N2" s="48"/>
-      <c r="O2" s="48"/>
-      <c r="P2" s="48"/>
+      <c r="N2" s="35"/>
+      <c r="O2" s="35"/>
+      <c r="P2" s="35"/>
       <c r="Q2" s="1"/>
       <c r="T2">
         <v>1</v>
@@ -6768,18 +6768,18 @@
     </row>
     <row r="3" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="34"/>
-      <c r="D3" s="34"/>
-      <c r="E3" s="34"/>
-      <c r="F3" s="34"/>
-      <c r="G3" s="34"/>
-      <c r="H3" s="34"/>
-      <c r="I3" s="34"/>
-      <c r="J3" s="34"/>
-      <c r="K3" s="34"/>
+      <c r="C3" s="32"/>
+      <c r="D3" s="32"/>
+      <c r="E3" s="32"/>
+      <c r="F3" s="32"/>
+      <c r="G3" s="32"/>
+      <c r="H3" s="32"/>
+      <c r="I3" s="32"/>
+      <c r="J3" s="32"/>
+      <c r="K3" s="32"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
@@ -6860,25 +6860,25 @@
     </row>
     <row r="6" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
-      <c r="B6" s="35" t="s">
+      <c r="B6" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="34"/>
-      <c r="D6" s="34"/>
-      <c r="E6" s="34"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="32"/>
+      <c r="C6" s="32"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="37"/>
       <c r="I6" s="1"/>
-      <c r="J6" s="50" t="s">
+      <c r="J6" s="38" t="s">
         <v>7</v>
       </c>
-      <c r="K6" s="34"/>
-      <c r="L6" s="34"/>
-      <c r="M6" s="34"/>
-      <c r="N6" s="34"/>
-      <c r="O6" s="34"/>
-      <c r="P6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32"/>
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="37"/>
       <c r="Q6" s="1"/>
       <c r="T6">
         <v>5</v>
@@ -6894,32 +6894,32 @@
     </row>
     <row r="7" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
-      <c r="B7" s="43">
+      <c r="B7" s="46">
         <f>'Store Total'!B4+'Store Total'!B5</f>
         <v>668</v>
       </c>
-      <c r="C7" s="34"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="34"/>
-      <c r="F7" s="53" t="s">
+      <c r="C7" s="32"/>
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="G7" s="34"/>
-      <c r="H7" s="32"/>
+      <c r="G7" s="32"/>
+      <c r="H7" s="37"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="40" t="str">
+      <c r="J7" s="49" t="str">
         <f>'Team Leaderboard'!$B$4</f>
         <v>Expert 01</v>
       </c>
-      <c r="K7" s="34"/>
-      <c r="L7" s="34"/>
-      <c r="M7" s="34"/>
-      <c r="N7" s="34"/>
-      <c r="O7" s="31">
+      <c r="K7" s="32"/>
+      <c r="L7" s="32"/>
+      <c r="M7" s="32"/>
+      <c r="N7" s="32"/>
+      <c r="O7" s="40">
         <f>'Team Leaderboard'!$E$4</f>
         <v>67</v>
       </c>
-      <c r="P7" s="32"/>
+      <c r="P7" s="37"/>
       <c r="Q7" s="1"/>
       <c r="T7">
         <v>6</v>
@@ -6935,30 +6935,30 @@
     </row>
     <row r="8" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1"/>
-      <c r="B8" s="39"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="36">
+      <c r="B8" s="43"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="54">
         <f>'Store Total'!C4+'Store Total'!C5</f>
         <v>645</v>
       </c>
-      <c r="G8" s="34"/>
-      <c r="H8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="37"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="40" t="str">
+      <c r="J8" s="49" t="str">
         <f>'Team Leaderboard'!$B$5</f>
         <v>Expert 07</v>
       </c>
-      <c r="K8" s="34"/>
-      <c r="L8" s="34"/>
-      <c r="M8" s="34"/>
-      <c r="N8" s="34"/>
-      <c r="O8" s="31">
+      <c r="K8" s="32"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="32"/>
+      <c r="N8" s="32"/>
+      <c r="O8" s="40">
         <f>'Team Leaderboard'!$E$5</f>
         <v>63</v>
       </c>
-      <c r="P8" s="32"/>
+      <c r="P8" s="37"/>
       <c r="Q8" s="1"/>
       <c r="T8">
         <v>7</v>
@@ -6974,27 +6974,27 @@
     </row>
     <row r="9" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1"/>
-      <c r="B9" s="39"/>
-      <c r="C9" s="34"/>
-      <c r="D9" s="34"/>
-      <c r="E9" s="34"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
+      <c r="E9" s="32"/>
       <c r="F9" s="9"/>
       <c r="G9" s="9"/>
       <c r="H9" s="5"/>
       <c r="I9" s="1"/>
-      <c r="J9" s="40" t="str">
+      <c r="J9" s="49" t="str">
         <f>'Team Leaderboard'!$B$6</f>
         <v>Expert 08</v>
       </c>
-      <c r="K9" s="34"/>
-      <c r="L9" s="34"/>
-      <c r="M9" s="34"/>
-      <c r="N9" s="34"/>
-      <c r="O9" s="31">
+      <c r="K9" s="32"/>
+      <c r="L9" s="32"/>
+      <c r="M9" s="32"/>
+      <c r="N9" s="32"/>
+      <c r="O9" s="40">
         <f>'Team Leaderboard'!$E$6</f>
         <v>62</v>
       </c>
-      <c r="P9" s="32"/>
+      <c r="P9" s="37"/>
       <c r="Q9" s="1"/>
       <c r="T9">
         <v>8</v>
@@ -7010,19 +7010,19 @@
     </row>
     <row r="10" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1"/>
-      <c r="B10" s="54" t="str">
+      <c r="B10" s="51" t="str">
         <f>IFERROR(TEXT(('Store Total'!B4+'Store Total'!B5)/('Store Total'!C4+'Store Total'!C5),"0%")&amp;" of goal","goal not set")</f>
         <v>104% of goal</v>
       </c>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="51" t="str">
+      <c r="C10" s="32"/>
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="41" t="str">
         <f>IFERROR(TEXT(('Store Total'!B4+'Store Total'!B5)-('Store Total'!C4+'Store Total'!C5),"+#,##0;-#,##0")&amp;" vs goal  ","")</f>
         <v xml:space="preserve">+23 vs goal  </v>
       </c>
-      <c r="G10" s="34"/>
-      <c r="H10" s="32"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="37"/>
       <c r="I10" s="1"/>
       <c r="J10" s="6"/>
       <c r="K10" s="10"/>
@@ -7046,30 +7046,30 @@
     </row>
     <row r="11" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1"/>
-      <c r="B11" s="49">
+      <c r="B11" s="36">
         <f>IFERROR(('Store Total'!B4+'Store Total'!B5)/('Store Total'!C4+'Store Total'!C5),0)</f>
         <v>1.0356589147286821</v>
       </c>
-      <c r="C11" s="34"/>
-      <c r="D11" s="34"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="34"/>
-      <c r="H11" s="32"/>
+      <c r="C11" s="32"/>
+      <c r="D11" s="32"/>
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32"/>
+      <c r="H11" s="37"/>
       <c r="I11" s="1"/>
-      <c r="J11" s="45" t="str">
+      <c r="J11" s="48" t="str">
         <f>'Team Leaderboard'!$B$15</f>
         <v>Expert 12</v>
       </c>
-      <c r="K11" s="34"/>
-      <c r="L11" s="34"/>
-      <c r="M11" s="34"/>
-      <c r="N11" s="34"/>
-      <c r="O11" s="52">
+      <c r="K11" s="32"/>
+      <c r="L11" s="32"/>
+      <c r="M11" s="32"/>
+      <c r="N11" s="32"/>
+      <c r="O11" s="44">
         <f>'Team Leaderboard'!$E$15</f>
         <v>38</v>
       </c>
-      <c r="P11" s="32"/>
+      <c r="P11" s="37"/>
       <c r="Q11" s="1"/>
       <c r="T11">
         <v>10</v>
@@ -7175,37 +7175,37 @@
     </row>
     <row r="15" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1"/>
-      <c r="B15" s="37" t="s">
+      <c r="B15" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="C15" s="34"/>
+      <c r="C15" s="32"/>
       <c r="D15" s="13" t="str">
         <f>TEXT('Store Total'!D4,"0%")</f>
         <v>105%</v>
       </c>
       <c r="E15" s="1"/>
-      <c r="F15" s="37" t="s">
+      <c r="F15" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="G15" s="34"/>
+      <c r="G15" s="32"/>
       <c r="H15" s="13" t="str">
         <f>TEXT('Store Total'!D5,"0%")</f>
         <v>94%</v>
       </c>
       <c r="I15" s="1"/>
-      <c r="J15" s="37" t="s">
+      <c r="J15" s="33" t="s">
         <v>11</v>
       </c>
-      <c r="K15" s="34"/>
+      <c r="K15" s="32"/>
       <c r="L15" s="13" t="str">
         <f>TEXT('Store Total'!D10,"0%")</f>
         <v>106%</v>
       </c>
       <c r="M15" s="1"/>
-      <c r="N15" s="37" t="s">
+      <c r="N15" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="O15" s="34"/>
+      <c r="O15" s="32"/>
       <c r="P15" s="13" t="str">
         <f>TEXT('Store Total'!D11,"0%")</f>
         <v>98%</v>
@@ -7225,33 +7225,33 @@
     </row>
     <row r="16" spans="1:22" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1"/>
-      <c r="B16" s="38">
+      <c r="B16" s="42">
         <f>'Store Total'!B4</f>
         <v>583</v>
       </c>
-      <c r="C16" s="34"/>
-      <c r="D16" s="32"/>
+      <c r="C16" s="32"/>
+      <c r="D16" s="37"/>
       <c r="E16" s="1"/>
-      <c r="F16" s="38">
+      <c r="F16" s="42">
         <f>'Store Total'!B5</f>
         <v>85</v>
       </c>
-      <c r="G16" s="34"/>
-      <c r="H16" s="32"/>
+      <c r="G16" s="32"/>
+      <c r="H16" s="37"/>
       <c r="I16" s="1"/>
-      <c r="J16" s="38">
+      <c r="J16" s="42">
         <f>'Store Total'!B10</f>
         <v>718</v>
       </c>
-      <c r="K16" s="34"/>
-      <c r="L16" s="32"/>
+      <c r="K16" s="32"/>
+      <c r="L16" s="37"/>
       <c r="M16" s="1"/>
-      <c r="N16" s="41">
+      <c r="N16" s="52">
         <f>'Store Total'!B11</f>
         <v>47740.969999999994</v>
       </c>
-      <c r="O16" s="34"/>
-      <c r="P16" s="32"/>
+      <c r="O16" s="32"/>
+      <c r="P16" s="37"/>
       <c r="Q16" s="1"/>
       <c r="T16">
         <v>15</v>
@@ -7267,21 +7267,21 @@
     </row>
     <row r="17" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1"/>
-      <c r="B17" s="39"/>
-      <c r="C17" s="34"/>
-      <c r="D17" s="32"/>
+      <c r="B17" s="43"/>
+      <c r="C17" s="32"/>
+      <c r="D17" s="37"/>
       <c r="E17" s="1"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="34"/>
-      <c r="H17" s="32"/>
+      <c r="F17" s="43"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="37"/>
       <c r="I17" s="1"/>
-      <c r="J17" s="39"/>
-      <c r="K17" s="34"/>
-      <c r="L17" s="32"/>
+      <c r="J17" s="43"/>
+      <c r="K17" s="32"/>
+      <c r="L17" s="37"/>
       <c r="M17" s="1"/>
-      <c r="N17" s="39"/>
-      <c r="O17" s="34"/>
-      <c r="P17" s="32"/>
+      <c r="N17" s="43"/>
+      <c r="O17" s="32"/>
+      <c r="P17" s="37"/>
       <c r="Q17" s="1"/>
       <c r="T17">
         <v>16</v>
@@ -7297,33 +7297,33 @@
     </row>
     <row r="18" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1"/>
-      <c r="B18" s="33">
+      <c r="B18" s="39">
         <f>'Store Total'!D4</f>
         <v>1.0504504504504504</v>
       </c>
-      <c r="C18" s="34"/>
-      <c r="D18" s="32"/>
+      <c r="C18" s="32"/>
+      <c r="D18" s="37"/>
       <c r="E18" s="1"/>
-      <c r="F18" s="33">
+      <c r="F18" s="39">
         <f>'Store Total'!D5</f>
         <v>0.94444444444444442</v>
       </c>
-      <c r="G18" s="34"/>
-      <c r="H18" s="32"/>
+      <c r="G18" s="32"/>
+      <c r="H18" s="37"/>
       <c r="I18" s="1"/>
-      <c r="J18" s="33">
+      <c r="J18" s="39">
         <f>'Store Total'!D10</f>
         <v>1.0637037037037036</v>
       </c>
-      <c r="K18" s="34"/>
-      <c r="L18" s="32"/>
+      <c r="K18" s="32"/>
+      <c r="L18" s="37"/>
       <c r="M18" s="1"/>
-      <c r="N18" s="33">
+      <c r="N18" s="39">
         <f>'Store Total'!D11</f>
         <v>0.98030739219712515</v>
       </c>
-      <c r="O18" s="34"/>
-      <c r="P18" s="32"/>
+      <c r="O18" s="32"/>
+      <c r="P18" s="37"/>
       <c r="Q18" s="1"/>
       <c r="T18">
         <v>17</v>
@@ -7429,37 +7429,37 @@
     </row>
     <row r="22" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1"/>
-      <c r="B22" s="37" t="s">
+      <c r="B22" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C22" s="34"/>
+      <c r="C22" s="32"/>
       <c r="D22" s="13" t="str">
         <f>TEXT('Store Total'!D7,"0%")</f>
         <v>96%</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="37" t="s">
+      <c r="F22" s="33" t="s">
         <v>14</v>
       </c>
-      <c r="G22" s="34"/>
+      <c r="G22" s="32"/>
       <c r="H22" s="13" t="str">
         <f>TEXT('Store Total'!D8,"0%")</f>
         <v>103%</v>
       </c>
       <c r="I22" s="1"/>
-      <c r="J22" s="37" t="s">
+      <c r="J22" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="K22" s="34"/>
+      <c r="K22" s="32"/>
       <c r="L22" s="13" t="str">
         <f>TEXT('Store Total'!D6,"0%")</f>
         <v>110%</v>
       </c>
       <c r="M22" s="1"/>
-      <c r="N22" s="37" t="s">
+      <c r="N22" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="O22" s="34"/>
+      <c r="O22" s="32"/>
       <c r="P22" s="13" t="str">
         <f>TEXT('Store Total'!D9,"0%")</f>
         <v>102%</v>
@@ -7479,33 +7479,33 @@
     </row>
     <row r="23" spans="1:22" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1"/>
-      <c r="B23" s="38">
+      <c r="B23" s="42">
         <f>'Store Total'!B7</f>
         <v>225</v>
       </c>
-      <c r="C23" s="34"/>
-      <c r="D23" s="32"/>
+      <c r="C23" s="32"/>
+      <c r="D23" s="37"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="38">
+      <c r="F23" s="42">
         <f>'Store Total'!B8</f>
         <v>31</v>
       </c>
-      <c r="G23" s="34"/>
-      <c r="H23" s="32"/>
+      <c r="G23" s="32"/>
+      <c r="H23" s="37"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="38">
+      <c r="J23" s="42">
         <f>'Store Total'!B6</f>
         <v>22</v>
       </c>
-      <c r="K23" s="34"/>
-      <c r="L23" s="32"/>
+      <c r="K23" s="32"/>
+      <c r="L23" s="37"/>
       <c r="M23" s="1"/>
-      <c r="N23" s="41">
+      <c r="N23" s="52">
         <f>'Store Total'!B9</f>
         <v>6702</v>
       </c>
-      <c r="O23" s="34"/>
-      <c r="P23" s="32"/>
+      <c r="O23" s="32"/>
+      <c r="P23" s="37"/>
       <c r="Q23" s="1"/>
       <c r="T23">
         <v>22</v>
@@ -7521,21 +7521,21 @@
     </row>
     <row r="24" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1"/>
-      <c r="B24" s="39"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="32"/>
+      <c r="B24" s="43"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="37"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="39"/>
-      <c r="G24" s="34"/>
-      <c r="H24" s="32"/>
+      <c r="F24" s="43"/>
+      <c r="G24" s="32"/>
+      <c r="H24" s="37"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="39"/>
-      <c r="K24" s="34"/>
-      <c r="L24" s="32"/>
+      <c r="J24" s="43"/>
+      <c r="K24" s="32"/>
+      <c r="L24" s="37"/>
       <c r="M24" s="1"/>
-      <c r="N24" s="39"/>
-      <c r="O24" s="34"/>
-      <c r="P24" s="32"/>
+      <c r="N24" s="43"/>
+      <c r="O24" s="32"/>
+      <c r="P24" s="37"/>
       <c r="Q24" s="1"/>
       <c r="T24">
         <v>23</v>
@@ -7551,33 +7551,33 @@
     </row>
     <row r="25" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="33">
+      <c r="B25" s="39">
         <f>'Store Total'!D7</f>
         <v>0.95744680851063835</v>
       </c>
-      <c r="C25" s="34"/>
-      <c r="D25" s="32"/>
+      <c r="C25" s="32"/>
+      <c r="D25" s="37"/>
       <c r="E25" s="1"/>
-      <c r="F25" s="33">
+      <c r="F25" s="39">
         <f>'Store Total'!D8</f>
         <v>1.0333333333333334</v>
       </c>
-      <c r="G25" s="34"/>
-      <c r="H25" s="32"/>
+      <c r="G25" s="32"/>
+      <c r="H25" s="37"/>
       <c r="I25" s="1"/>
-      <c r="J25" s="33">
+      <c r="J25" s="39">
         <f>'Store Total'!D6</f>
         <v>1.1000000000000001</v>
       </c>
-      <c r="K25" s="34"/>
-      <c r="L25" s="32"/>
+      <c r="K25" s="32"/>
+      <c r="L25" s="37"/>
       <c r="M25" s="1"/>
-      <c r="N25" s="33">
+      <c r="N25" s="39">
         <f>'Store Total'!D9</f>
         <v>1.0154545454545454</v>
       </c>
-      <c r="O25" s="34"/>
-      <c r="P25" s="32"/>
+      <c r="O25" s="32"/>
+      <c r="P25" s="37"/>
       <c r="Q25" s="1"/>
       <c r="T25">
         <v>24</v>
@@ -7683,19 +7683,19 @@
     </row>
     <row r="29" spans="1:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1"/>
-      <c r="B29" s="46" t="s">
+      <c r="B29" s="31" t="s">
         <v>17</v>
       </c>
-      <c r="C29" s="34"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="34"/>
-      <c r="F29" s="34"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
-      <c r="K29" s="34"/>
-      <c r="L29" s="34"/>
+      <c r="C29" s="32"/>
+      <c r="D29" s="32"/>
+      <c r="E29" s="32"/>
+      <c r="F29" s="32"/>
+      <c r="G29" s="32"/>
+      <c r="H29" s="32"/>
+      <c r="I29" s="32"/>
+      <c r="J29" s="32"/>
+      <c r="K29" s="32"/>
+      <c r="L29" s="32"/>
       <c r="M29" s="10"/>
       <c r="N29" s="10"/>
       <c r="O29" s="10"/>
@@ -8074,6 +8074,34 @@
     </row>
   </sheetData>
   <mergeCells count="44">
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="N18:P18"/>
+    <mergeCell ref="B6:H6"/>
+    <mergeCell ref="F8:H8"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="O9:P9"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="B16:D17"/>
+    <mergeCell ref="J25:L25"/>
+    <mergeCell ref="J9:N9"/>
+    <mergeCell ref="J23:L24"/>
+    <mergeCell ref="F16:H17"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="N16:P17"/>
+    <mergeCell ref="J18:L18"/>
+    <mergeCell ref="B23:D24"/>
+    <mergeCell ref="N23:P24"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="B7:E9"/>
+    <mergeCell ref="B3:K3"/>
+    <mergeCell ref="J11:N11"/>
+    <mergeCell ref="J7:N7"/>
+    <mergeCell ref="F7:H7"/>
+    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="J8:N8"/>
     <mergeCell ref="B29:L29"/>
     <mergeCell ref="F22:G22"/>
     <mergeCell ref="M2:P2"/>
@@ -8090,34 +8118,6 @@
     <mergeCell ref="B15:C15"/>
     <mergeCell ref="J16:L17"/>
     <mergeCell ref="N15:O15"/>
-    <mergeCell ref="B2:I2"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="B7:E9"/>
-    <mergeCell ref="B3:K3"/>
-    <mergeCell ref="J11:N11"/>
-    <mergeCell ref="J7:N7"/>
-    <mergeCell ref="F7:H7"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="J8:N8"/>
-    <mergeCell ref="B22:C22"/>
-    <mergeCell ref="O9:P9"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="B16:D17"/>
-    <mergeCell ref="J25:L25"/>
-    <mergeCell ref="J9:N9"/>
-    <mergeCell ref="J23:L24"/>
-    <mergeCell ref="F16:H17"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="N16:P17"/>
-    <mergeCell ref="J18:L18"/>
-    <mergeCell ref="B23:D24"/>
-    <mergeCell ref="N23:P24"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="F18:H18"/>
-    <mergeCell ref="N18:P18"/>
-    <mergeCell ref="B6:H6"/>
-    <mergeCell ref="F8:H8"/>
   </mergeCells>
   <conditionalFormatting sqref="B11">
     <cfRule type="dataBar" priority="1">
@@ -9409,13 +9409,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -11822,13 +11822,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -13897,13 +13897,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -16206,13 +16206,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -18463,13 +18463,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -20694,13 +20694,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -22899,13 +22899,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -25130,13 +25130,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -27283,13 +27283,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -29644,13 +29644,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -32445,13 +32445,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -34494,13 +34494,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -36699,13 +36699,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -38878,13 +38878,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -40927,13 +40927,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -43002,13 +43002,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -45155,13 +45155,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -47568,13 +47568,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -49877,13 +49877,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -52030,13 +52030,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -55339,13 +55339,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -57648,13 +57648,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -59671,13 +59671,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -62006,13 +62006,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -64315,13 +64315,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -66598,13 +66598,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -68959,13 +68959,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -71584,13 +71584,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -73607,13 +73607,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -75942,13 +75942,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
@@ -78277,13 +78277,13 @@
         <f>IF(COUNTA($A$4:$A$63)&lt;&gt;COUNTA($D$4:$D$63),"!! rows are missing a Mobile Expert — they still count in the store total but not against any person","all rows assigned")</f>
         <v>all rows assigned</v>
       </c>
-      <c r="R18" s="34"/>
-      <c r="S18" s="34"/>
-      <c r="T18" s="34"/>
-      <c r="U18" s="34"/>
-      <c r="V18" s="34"/>
-      <c r="W18" s="34"/>
-      <c r="X18" s="34"/>
+      <c r="R18" s="32"/>
+      <c r="S18" s="32"/>
+      <c r="T18" s="32"/>
+      <c r="U18" s="32"/>
+      <c r="V18" s="32"/>
+      <c r="W18" s="32"/>
+      <c r="X18" s="32"/>
     </row>
     <row r="19" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">

</xml_diff>